<commit_message>
refactor: rename cross-chain scope to module B
</commit_message>
<xml_diff>
--- a/module1-basic-testing/docs/test-cases.xlsx
+++ b/module1-basic-testing/docs/test-cases.xlsx
@@ -1515,7 +1515,7 @@
     <row r="16" ht="18.9" customHeight="1">
       <c r="B16" s="4" t="inlineStr">
         <is>
-          <t>本批次采用传统测试方法，当前范围为模块 A 认证与访问控制、模块 C 跨链任务状态控制。模块 B 文件上传与完整性验证暂缓。</t>
+          <t>本批次采用传统测试方法，当前范围为模块 A 认证与访问控制、模块 B 跨链任务状态控制。</t>
         </is>
       </c>
       <c r="C16" s="14" t="n"/>
@@ -1609,7 +1609,7 @@
       </c>
       <c r="E20" s="11" t="inlineStr">
         <is>
-          <t>建立 A+C 测试基线</t>
+          <t>建立 A+B 测试基线</t>
         </is>
       </c>
       <c r="F20" s="11" t="n"/>
@@ -3894,7 +3894,7 @@
     <row r="25" ht="58" customHeight="1">
       <c r="A25" s="68" t="inlineStr">
         <is>
-          <t>C-001</t>
+          <t>B-001</t>
         </is>
       </c>
       <c r="B25" s="68" t="inlineStr">
@@ -3962,7 +3962,7 @@
     <row r="26" ht="58" customHeight="1">
       <c r="A26" s="68" t="inlineStr">
         <is>
-          <t>C-002</t>
+          <t>B-002</t>
         </is>
       </c>
       <c r="B26" s="68" t="inlineStr">
@@ -4030,7 +4030,7 @@
     <row r="27" ht="58" customHeight="1">
       <c r="A27" s="68" t="inlineStr">
         <is>
-          <t>C-003</t>
+          <t>B-003</t>
         </is>
       </c>
       <c r="B27" s="68" t="inlineStr">
@@ -4098,7 +4098,7 @@
     <row r="28" ht="58" customHeight="1">
       <c r="A28" s="68" t="inlineStr">
         <is>
-          <t>C-004</t>
+          <t>B-004</t>
         </is>
       </c>
       <c r="B28" s="68" t="inlineStr">
@@ -4166,7 +4166,7 @@
     <row r="29" ht="58" customHeight="1">
       <c r="A29" s="68" t="inlineStr">
         <is>
-          <t>C-005</t>
+          <t>B-005</t>
         </is>
       </c>
       <c r="B29" s="68" t="inlineStr">
@@ -4234,7 +4234,7 @@
     <row r="30" ht="58" customHeight="1">
       <c r="A30" s="68" t="inlineStr">
         <is>
-          <t>C-006</t>
+          <t>B-006</t>
         </is>
       </c>
       <c r="B30" s="68" t="inlineStr">
@@ -4302,7 +4302,7 @@
     <row r="31" ht="58" customHeight="1">
       <c r="A31" s="68" t="inlineStr">
         <is>
-          <t>C-007</t>
+          <t>B-007</t>
         </is>
       </c>
       <c r="B31" s="68" t="inlineStr">
@@ -4370,7 +4370,7 @@
     <row r="32" ht="58" customHeight="1">
       <c r="A32" s="68" t="inlineStr">
         <is>
-          <t>C-008</t>
+          <t>B-008</t>
         </is>
       </c>
       <c r="B32" s="68" t="inlineStr">
@@ -4438,7 +4438,7 @@
     <row r="33" ht="58" customHeight="1">
       <c r="A33" s="68" t="inlineStr">
         <is>
-          <t>C-009</t>
+          <t>B-009</t>
         </is>
       </c>
       <c r="B33" s="68" t="inlineStr">

</xml_diff>